<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.002-04 Raphaël et la tour de cubes
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.002-04.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.002-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, après-midi</t>
+          <t>salon, après-midi, cubes, tour, chat, fauteuil, soleil, bois, pain, bol, pull</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Le chat passe. La tour de cubes de Raphaël tombe. Il dit qu'il est triste. Il demande un câlin. Une petite tour recommence.</t>
+          <t>Le chat frotte le dossier, puis s'en va. Sur le tissu, un éclat de fauteuil luit. Raphaël veut la tour, maintenant. La queue du chat balaie les cubes. Poitrine trop vite. Sourire parti. Yeux chauds. Papa s'accroupit. Je suis triste. Un câlin. Merci vécu. Deuxième ruse : le chat revient, un cube roule. Il refuse de foncer. Une petite tour recommence. Un éclat de fauteuil tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le rideau se lève un peu. Un carré de soleil est sur le plancher. Le bois est tiède sous les pieds. Dans la cuisine, le bol du chat tinte. Ça sent le pain encore chaud. Des cubes bleus attendent près du tapis. Raphaël, tu as tes cubes ? Oui. Les bleus et les jaunes. Je reste près du tapis, d'accord ? D'accord, papa. En ce moment, Raphaël pose un cube. Puis un autre, tout doucement. La tour monte, bleue et jaune. Elle est haute, papa. Elle est haute, oui. Le chat passe, tout près. Sa queue balaie le tapis. Les cubes tombent. Ils font un bruit sourd. Ma tour... Parce que la tour est tombée. Raphaël sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Raphaël pleure un peu. Les larmes coulent. Elles sont chaudes. Je t'écoute, Raphaël. Je veux un câlin. Viens. Un câlin. Papa ouvre les bras. Raphaël se blottit contre papa. Le câlin est chaud. Le pull de papa sent le pain. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Raphaël. Le câlin aide. Oui. Le câlin aide. Plus tard, papa pose un cube bleu. Un cube pour toi. Raphaël pose un cube jaune. Un cube pour moi. Une petite tour recommence. Elle est petite. Elle est petite. Elle est à nous. Tu veux encore un cube ? Encore un jaune. Raphaël souffle. Ses épaules se desserrent. Le carré de soleil a un peu bougé.</t>
+          <t>Le chat frotte le dossier, puis s'en va. Il part, papa. Tu l'as vu, le chat ? Oui, papa. Le dossier du fauteuil reste chaud, sous le soleil. Il est chaud, maman. Tu le touches, le dossier ? Oui. Le tissu sent le soleil d'après-midi. Ça sent le chaud. Dans la cuisine, le bol du chat tinte. Il boit, maman. Tu l'entends, le bol ? Oui, maman. Des cubes bleus attendent près du fauteuil. Les bleus et les jaunes ! Tu as tes cubes, Raphaël ? Oui, papa. Sur le tissu, un éclat de fauteuil luit. Il brille, maman. Tu le vois, le petit point ? Oui, un point clair. Le soleil le touche. Un cube jaune pèse dans sa main. Il est lisse. En ce moment, Raphaël pose un cube. Je veux la tour, maintenant ! Tout de suite ? Oui, papa. Il pose un cube trop vite, trop haut. Plus haut ! Puis un autre, plus haut que le premier. Elle est haute, papa. Elle est haute, oui. La tour penche un peu vers le fauteuil. Elle tient ! Tes mains vont trop vite, Raphaël ? Un peu. Le chat revient du bol, tout près. Sa queue balaie le bas de la tour. Les cubes tombent sur le bois. Ma tour ! Ils font un bruit sourd, près des pieds. Raphaël reste surpris, les mains ouvertes. Sa gorge se serre d'un coup. Oh. Ses yeux deviennent chauds. Une larme tombe sur le bois. Je suis triste. Raphaël pleure un peu, sans crier. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se heurtent. Tu as les yeux chauds, Raphaël ? Oui, papa. Sa poitrine va trop vite. Papa s'accroupit à la même hauteur. Je veux un câlin. Viens. Papa ouvre les bras, tout près du fauteuil. Raphaël se blottit contre papa. Le câlin est chaud, près du cou. Ton pull sent le pain. L'éclat de fauteuil tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le rideau se lève un peu. Un carré de soleil est sur le plancher. Le bois est tiède sous les pieds. Dans la cuisine, le bol du chat tinte. Ça sent le pain encore chaud. Des cubes bleus attendent près du tapis. Raphaël, tu as tes cubes ? Oui. Les bleus et les jaunes. Je reste près du tapis, d'accord ? D'accord, papa. En ce moment, Raphaël pose un cube. Puis un autre, tout doucement. La tour monte, bleue et jaune. Elle est haute, papa. Elle est haute, oui. Le chat passe, tout près. Sa queue balaie le tapis. Les cubes tombent. Ils font un bruit sourd. Ma tour... Parce que la tour est tombée. Raphaël sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Raphaël pleure un peu. Les larmes coulent. Elles sont chaudes. Je t'écoute, Raphaël. Je veux un câlin. Viens. Un câlin. Papa ouvre les bras. Raphaël se blottit contre papa. Le câlin est chaud. Le pull de papa sent le pain. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Raphaël. Le câlin aide. Oui. Le câlin aide. Plus tard, papa pose un cube bleu. Un cube pour toi. Raphaël pose un cube jaune. Un cube pour moi. Une petite tour recommence. Elle est petite. Elle est petite. Elle est à nous. Tu veux encore un cube ? Encore un jaune. Raphaël souffle. Ses épaules se desserrent. Le carré de soleil a un peu bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le chat frotte le dossier, puis s'en va. Il part, papa. Tu l'as vu, le chat ? Oui, papa. Le dossier du fauteuil reste chaud, sous le soleil. Il est chaud, maman. Tu le touches, le dossier ? Oui. Le tissu sent le soleil d'après-midi. Ça sent le chaud. Dans la cuisine, le bol du chat tinte. Il boit, maman. Tu l'entends, le bol ? Oui, maman. Des cubes bleus attendent près du fauteuil. Les bleus et les jaunes ! Tu as tes cubes, Raphaël ? Oui, papa. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de fauteuil&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un point clair. Le soleil le touche. Un cube jaune pèse dans sa main. Il est lisse. En ce moment, Raphaël pose un cube. Je veux la tour, maintenant ! Tout de suite ? Oui, papa. Il pose un cube trop vite, trop haut. Plus haut ! Puis un autre, plus haut que le premier. Elle est haute, papa. Elle est haute, oui. La tour penche un peu vers le fauteuil. Elle tient ! Tes mains vont trop vite, Raphaël ? Un peu. Le chat revient du bol, tout près. Sa queue balaie le bas de la tour. Les cubes tombent sur le bois. Ma tour ! Ils font un bruit sourd, près des pieds. Raphaël reste surpris, les mains ouvertes. Sa gorge se serre d'un coup. Oh. Ses yeux deviennent chauds. Une larme tombe sur le bois. Je suis triste. Raphaël pleure un peu, sans crier. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se heurtent. Tu as les yeux chauds, Raphaël ? Oui, papa. Sa poitrine va trop vite. Papa s'accroupit à la même hauteur. Je veux un câlin. Viens. Papa ouvre les bras, tout près du fauteuil. Raphaël se blottit contre papa. Le câlin est chaud, près du cou. Ton pull sent le pain. L'éclat de fauteuil tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Mateo construit une tour dans le salon. Les cubes sont bleus et jaunes. La tour est haute. Le chat passe. Les cubes tombent. Ils font un bruit sourd. Mateo sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Mateo dit : je suis &lt;emphasis&gt;triste&lt;/emphasis&gt;. Papa arrive près de lui. Papa dit : pleurer est permis. Mateo pleure un peu. Les larmes coulent. Puis Mateo dit : je veux un câlin. Papa ouvre les bras. Mateo se blottit contre papa. Le câlin est chaud. Parce que la tour est tombée, Mateo est triste. Être triste, c'est permis. Plus tard, papa pose un cube. Mateo pose un cube. Une petite tour recommence. Mateo souffle. Ses épaules se desserrent. [pause]</t>
+          <t>Le chat frotte le dossier, puis s'en va. Il part, papa. Tu l'as vu, le chat ? Oui, papa. Le dossier du fauteuil reste chaud, sous le soleil. Il est chaud, maman. Tu le touches, le dossier ? Oui. Le tissu sent le soleil d'après-midi. Ça sent le chaud. Dans la cuisine, le bol du chat tinte. Il boit, maman. Tu l'entends, le bol ? Oui, maman. Des cubes bleus attendent près du fauteuil. Les bleus et les jaunes ! Tu as tes cubes, Raphaël ? Oui, papa. Sur le tissu, un &lt;emphasis&gt;éclat de fauteuil&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un point clair. Le soleil le touche. Un cube jaune pèse dans sa main. Il est lisse. En ce moment, Raphaël pose un cube. Je veux la tour, maintenant ! Tout de suite ? Oui, papa. Il pose un cube trop vite, trop haut. Plus haut ! Puis un autre, plus haut que le premier. Elle est haute, papa. Elle est haute, oui. La tour penche un peu vers le fauteuil. Elle tient ! Tes mains vont trop vite, Raphaël ? Un peu. Le chat revient du bol, tout près. Sa queue balaie le bas de la tour. Les cubes tombent sur le bois. Ma tour ! Ils font un bruit sourd, près des pieds. Raphaël reste surpris, les mains ouvertes. Sa gorge se serre d'un coup. Oh. Ses yeux deviennent chauds. Une larme tombe sur le bois. Je suis triste. Raphaël pleure un peu, sans crier. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se heurtent. Tu as les yeux chauds, Raphaël ? Oui, papa. Sa poitrine va trop vite. Papa s'accroupit à la même hauteur. Je veux un câlin. Viens. Papa ouvre les bras, tout près du fauteuil. Raphaël se blottit contre papa. Le câlin est chaud, près du cou. Ton pull sent le pain. L'éclat de fauteuil tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>éclat de fauteuil</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,62 +1321,81 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis tristesse; intensite=2; destinataire=enfant; sous_texte=il_veut_la_tour_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le rideau se lève un peu.
-narrateur|Un carré de soleil est sur le plancher.
-narrateur|Le bois est tiède sous les pieds.
+          <t>narrateur|Le chat frotte le dossier, puis s'en va.
+enfant-m|Il part, papa.
+papa|Tu l'as vu, le chat ?
+enfant-m|Oui, papa.
+narrateur|Le dossier du fauteuil reste chaud, sous le soleil.
+enfant-m|Il est chaud, maman.
+maman|Tu le touches, le dossier ?
+enfant-m|Oui.
+narrateur|Le tissu sent le soleil d'après-midi.
+enfant-m|Ça sent le chaud.
 narrateur|Dans la cuisine, le bol du chat tinte.
-narrateur|Ça sent le pain encore chaud.
-narrateur|Des cubes bleus attendent près du tapis.
-maman|Raphaël, tu as tes cubes ?
-enfant-m|Oui. Les bleus et les jaunes.
-papa|Je reste près du tapis, d'accord ?
-enfant-m|D'accord, papa.
+enfant-m|Il boit, maman.
+maman|Tu l'entends, le bol ?
+enfant-m|Oui, maman.
+narrateur|Des cubes bleus attendent près du fauteuil.
+enfant-m|Les bleus et les jaunes !
+papa|Tu as tes cubes, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Sur le tissu, un éclat de fauteuil luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un point clair.
+papa|Le soleil le touche.
+narrateur|Un cube jaune pèse dans sa main.
+enfant-m|Il est lisse.
 narrateur|En ce moment, Raphaël pose un cube.
-narrateur|Puis un autre, tout doucement.
-narrateur|La tour monte, bleue et jaune.
+enfant-m|Je veux la tour, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Il pose un cube trop vite, trop haut.
+enfant-m|Plus haut !
+narrateur|Puis un autre, plus haut que le premier.
 enfant-m|Elle est haute, papa.
 papa|Elle est haute, oui.
-narrateur|Le chat passe, tout près.
-narrateur|Sa queue balaie le tapis.
-narrateur|Les cubes tombent.
-narrateur|Ils font un bruit sourd.
-enfant-m|Ma tour...
-narrateur|Parce que la tour est tombée.
-narrateur|Raphaël sent sa gorge serrée.
+narrateur|La tour penche un peu vers le fauteuil.
+enfant-m|Elle tient !
+maman|Tes mains vont trop vite, Raphaël ?
+enfant-m|Un peu.
+narrateur|Le chat revient du bol, tout près.
+narrateur|Sa queue balaie le bas de la tour.
+narrateur|Les cubes tombent sur le bois.
+enfant-m|Ma tour !
+narrateur|Ils font un bruit sourd, près des pieds.
+narrateur|Raphaël reste surpris, les mains ouvertes.
+narrateur|Sa gorge se serre d'un coup.
+enfant-m|Oh.
 narrateur|Ses yeux deviennent chauds.
-narrateur|Une larme tombe.
+narrateur|Une larme tombe sur le bois.
 enfant-m|Je suis triste.
-papa|Tu es triste. C'est permis.
-papa|Pleurer est permis.
-narrateur|Raphaël pleure un peu.
-narrateur|Les larmes coulent. Elles sont chaudes.
-maman|Je t'écoute, Raphaël.
+narrateur|Raphaël pleure un peu, sans crier.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se heurtent.
+papa|Tu as les yeux chauds, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Sa poitrine va trop vite.
+narrateur|Papa s'accroupit à la même hauteur.
 enfant-m|Je veux un câlin.
-papa|Viens. Un câlin.
-narrateur|Papa ouvre les bras.
+papa|Viens.
+narrateur|Papa ouvre les bras, tout près du fauteuil.
 narrateur|Raphaël se blottit contre papa.
-narrateur|Le câlin est chaud.
-narrateur|Le pull de papa sent le pain.
-maman|Tu as dit : je suis triste.
-maman|Bravo. Tu as demandé un câlin.
-papa|Pleurer est permis, Raphaël.
-enfant-m|Le câlin aide.
-papa|Oui. Le câlin aide.
-narrateur|Plus tard, papa pose un cube bleu.
-papa|Un cube pour toi.
-narrateur|Raphaël pose un cube jaune.
-enfant-m|Un cube pour moi.
-narrateur|Une petite tour recommence.
-enfant-m|Elle est petite.
-papa|Elle est petite. Elle est à nous.
-maman|Tu veux encore un cube ?
-enfant-m|Encore un jaune.
-narrateur|Raphaël souffle.
-narrateur|Ses épaules se desserrent.
-narrateur|Le carré de soleil a un peu bougé.</t>
+narrateur|Le câlin est chaud, près du cou.
+enfant-m|Ton pull sent le pain.
+narrateur|L'éclat de fauteuil tremble, puis tient.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>cubes_tombent,chat</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1427,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a les yeux chauds. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Raphaël&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Mateo a les yeux chauds. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Raphaël&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1438,7 +1457,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Mateo peut demander un câlin. Que dit-il ?</t>
+          <t>Raphaël peut demander un câlin. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1476,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1487,7 +1506,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1502,34 +1521,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Raphaël</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1544,22 +1567,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=raphael_a_les_yeux_chauds_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a les yeux chauds. Que dit-il ?</t>
+          <t>narrateur|Raphaël a les yeux chauds.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Le câlin aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Papa le serre, sans se presser. Le tapis est doux sous les genoux.</t>
+          <t>Raphaël reste contre papa, un moment. La tour, maintenant. Les mots se bousculent dans sa bouche. Je la refais. Raphaël avance les mains, trop vite. Puis il s'arrête. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle, près du fauteuil. Il observe les cubes, un instant. Ils sont par terre. Tu restes un peu, Raphaël ? Oui, papa. Merci, Raphaël. Papa reste à la même hauteur. Le câlin est tiède, sous les bras. Il est chaud. La poitrine de Raphaël ralentit un peu. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Maman essuie une larme du pouce. Le soleil touche le dossier ? Oui, maman. Le ventre de Raphaël se desserre. On pose un cube, sans se presser ? Oui, papa. Raphaël tient le pull de papa. Je reste un peu. Ils se baissent, sans se bousculer. Un bleu, papa. On le pose, sans se presser.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Le câlin aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Papa le serre, sans se presser. Le tapis est doux sous les genoux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël reste contre papa, un moment. La tour, maintenant. Les mots se bousculent dans sa bouche. Je la refais. Raphaël avance les mains, trop vite. Puis il s'arrête. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle, près du fauteuil. Il observe les cubes, un instant. Ils sont par terre. Tu restes un peu, Raphaël ? Oui, papa. Merci, Raphaël. Papa reste à la même hauteur. Le &lt;emphasis level="moderate"&gt;câlin&lt;/emphasis&gt; est tiède, sous les bras. Il est chaud. La poitrine de Raphaël ralentit un peu. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Maman essuie une larme du pouce. Le soleil touche le dossier ? Oui, maman. Le ventre de Raphaël se desserre. On pose un cube, sans se presser ? Oui, papa. Raphaël tient le pull de papa. Je reste un peu. Ils se baissent, sans se bousculer. Un bleu, papa. On le pose, sans se presser.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Mateo a nommé : &lt;emphasis&gt;triste&lt;/emphasis&gt;. Pleurer est permis. Un câlin de papa aide. [pause]</t>
+          <t>Raphaël reste contre papa, un moment. La tour, maintenant. Les mots se bousculent dans sa bouche. Je la refais. Raphaël avance les mains, trop vite. Puis il s'arrête. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle, près du fauteuil. Il observe les cubes, un instant. Ils sont par terre. Tu restes un peu, Raphaël ? Oui, papa. Merci, Raphaël. Papa reste à la même hauteur. Le &lt;emphasis&gt;câlin&lt;/emphasis&gt; est tiède, sous les bras. Il est chaud. La poitrine de Raphaël ralentit un peu. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Maman essuie une larme du pouce. Le soleil touche le dossier ? Oui, maman. Le ventre de Raphaël se desserre. On pose un cube, sans se presser ? Oui, papa. Raphaël tient le pull de papa. Je reste un peu. Ils se baissent, sans se bousculer. Un bleu, papa. On le pose, sans se presser. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1654,7 +1678,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1701,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>câlin</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1691,16 +1715,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1725,20 +1749,43 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=il_demande_un_calin_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël sèche une larme avec sa manche.
-enfant-m|Je suis triste.
-papa|Oui. Et pleurer est permis.
-papa|Le câlin aide.
-maman|Bravo. Tu as dit ce que tu sentais.
-maman|Tu veux encore un câlin ?
-enfant-m|Encore un peu.
-narrateur|Papa le serre, sans se presser.
-narrateur|Le tapis est doux sous les genoux.</t>
+          <t>narrateur|Raphaël reste contre papa, un moment.
+enfant-m|La tour, maintenant.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Je la refais.
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle, près du fauteuil.
+narrateur|Il observe les cubes, un instant.
+enfant-m|Ils sont par terre.
+papa|Tu restes un peu, Raphaël ?
+enfant-m|Oui, papa.
+papa|Merci, Raphaël.
+narrateur|Papa reste à la même hauteur.
+maman|Le câlin est tiède, sous les bras.
+enfant-m|Il est chaud.
+narrateur|La poitrine de Raphaël ralentit un peu.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près des cubes ?
+enfant-m|Oui.
+narrateur|Maman essuie une larme du pouce.
+maman|Le soleil touche le dossier ?
+enfant-m|Oui, maman.
+narrateur|Le ventre de Raphaël se desserre.
+papa|On pose un cube, sans se presser ?
+enfant-m|Oui, papa.
+narrateur|Raphaël tient le pull de papa.
+enfant-m|Je reste un peu.
+narrateur|Ils se baissent, sans se bousculer.
+enfant-m|Un bleu, papa.
+papa|On le pose, sans se presser.</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1812,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël pose un dernier cube. La petite tour tient. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. On laisse la tour jusqu'au goûter ? Oui. Tout près. Papa reste près de lui. Le chat se couche au soleil.</t>
+          <t>Maman pousse un cube bleu près du bois. Le bois est un peu poudreux. La tour, maintenant ! Raphaël prend trop de cubes, tout de suite. Un cube jaune glisse de sa main. Il glisse ! Le cube continue de rouler vers le fauteuil. Il roule ! Le chat revient vers les cubes. Sa queue passe tout près du bois. Le chat ! La petite tour penche vers le dossier. Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. J'attends. Il observe les cubes, un instant. Il écoute le salon, près du fauteuil. Sur le tissu, un éclat de fauteuil luit. Là, sur le tissu. On tient le cube ? Oui, papa. Le cube jaune s'arrête contre le dossier. Raphaël le prend, sans se presser. Il est lisse. Le chat reste près de nous ? Oui, papa. Le chat s'assoit, loin des cubes. Il regarde. Tu poses le cube, Raphaël ? Oui, maman. Papa pose un cube bleu. Un cube pour toi. Raphaël pose un cube jaune. Un cube pour moi. Une petite tour recommence, près du fauteuil. Elle est petite. Elle est petite, à nous. Tu vois le point, Raphaël ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. On reste ici, Raphaël ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël pose un dernier cube. La petite tour tient. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. On laisse la tour jusqu'au goûter ? Oui. Tout près. Papa reste près de lui. Le chat se couche au soleil.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse un cube bleu près du bois. Le bois est un peu poudreux. La tour, maintenant ! Raphaël prend trop de cubes, tout de suite. Un cube jaune glisse de sa main. Il glisse ! Le cube continue de rouler vers le fauteuil. Il roule ! Le chat revient vers les cubes. Sa queue passe tout près du bois. Le chat ! La petite tour penche vers le dossier. Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. J'attends. Il observe les cubes, un instant. Il écoute le salon, près du fauteuil. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de fauteuil&lt;/emphasis&gt; luit. Là, sur le tissu. On tient le cube ? Oui, papa. Le cube jaune s'arrête contre le dossier. Raphaël le prend, sans se presser. Il est lisse. Le chat reste près de nous ? Oui, papa. Le chat s'assoit, loin des cubes. Il regarde. Tu poses le cube, Raphaël ? Oui, maman. Papa pose un cube bleu. Un cube pour toi. Raphaël pose un cube jaune. Un cube pour moi. Une petite tour recommence, près du fauteuil. Elle est petite. Elle est petite, à nous. Tu vois le point, Raphaël ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. On reste ici, Raphaël ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Mateo pose un dernier cube. Papa reste près de lui. [pause]</t>
+          <t>Maman pousse un cube bleu près du bois. Le bois est un peu poudreux. La tour, maintenant ! Raphaël prend trop de cubes, tout de suite. Un cube jaune glisse de sa main. Il glisse ! Le cube continue de rouler vers le fauteuil. Il roule ! Le chat revient vers les cubes. Sa queue passe tout près du bois. Le chat ! La petite tour penche vers le dossier. Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. J'attends. Il observe les cubes, un instant. Il écoute le salon, près du fauteuil. Sur le tissu, un &lt;emphasis&gt;éclat de fauteuil&lt;/emphasis&gt; luit. Là, sur le tissu. On tient le cube ? Oui, papa. Le cube jaune s'arrête contre le dossier. Raphaël le prend, sans se presser. Il est lisse. Le chat reste près de nous ? Oui, papa. Le chat s'assoit, loin des cubes. Il regarde. Tu poses le cube, Raphaël ? Oui, maman. Papa pose un cube bleu. Un cube pour toi. Raphaël pose un cube jaune. Un cube pour moi. Une petite tour recommence, près du fauteuil. Elle est petite. Elle est petite, à nous. Tu vois le point, Raphaël ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. On reste ici, Raphaël ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1869,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,10 +1877,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1854,28 +1901,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de fauteuil</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1884,10 +1935,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1898,18 +1949,64 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=chat_revient_cube_roule_il_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël pose un dernier cube.
-narrateur|La petite tour tient.
-papa|Tu as bien demandé le câlin.
-enfant-m|Je suis moins triste.
-maman|Le câlin est encore là.
-maman|On laisse la tour jusqu'au goûter ?
-enfant-m|Oui. Tout près.
-narrateur|Papa reste près de lui.
-narrateur|Le chat se couche au soleil.</t>
+          <t>narrateur|Maman pousse un cube bleu près du bois.
+narrateur|Le bois est un peu poudreux.
+enfant-m|La tour, maintenant !
+narrateur|Raphaël prend trop de cubes, tout de suite.
+narrateur|Un cube jaune glisse de sa main.
+enfant-m|Il glisse !
+narrateur|Le cube continue de rouler vers le fauteuil.
+enfant-m|Il roule !
+narrateur|Le chat revient vers les cubes.
+narrateur|Sa queue passe tout près du bois.
+enfant-m|Le chat !
+narrateur|La petite tour penche vers le dossier.
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+enfant-m|J'attends.
+narrateur|Il observe les cubes, un instant.
+narrateur|Il écoute le salon, près du fauteuil.
+narrateur|Sur le tissu, un éclat de fauteuil luit.
+enfant-m|Là, sur le tissu.
+papa|On tient le cube ?
+enfant-m|Oui, papa.
+narrateur|Le cube jaune s'arrête contre le dossier.
+narrateur|Raphaël le prend, sans se presser.
+enfant-m|Il est lisse.
+papa|Le chat reste près de nous ?
+enfant-m|Oui, papa.
+narrateur|Le chat s'assoit, loin des cubes.
+enfant-m|Il regarde.
+maman|Tu poses le cube, Raphaël ?
+enfant-m|Oui, maman.
+narrateur|Papa pose un cube bleu.
+papa|Un cube pour toi.
+narrateur|Raphaël pose un cube jaune.
+enfant-m|Un cube pour moi.
+narrateur|Une petite tour recommence, près du fauteuil.
+enfant-m|Elle est petite.
+papa|Elle est petite, à nous.
+papa|Tu vois le point, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Les cubes tiennent, l'un sur l'autre.
+enfant-m|C'est plus facile.
+papa|On reste ici, Raphaël ?
+enfant-m|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>chat,cubes</t>
         </is>
       </c>
     </row>
@@ -1936,17 +2033,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Raphaël.</t>
+          <t>Ils restent près du fauteuil. Maman essuie un peu de bois. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près de la tour. Raphaël tapote le tissu du doigt. Il a une trace de soleil. Tu la vois, la trace ? Oui, maman. La petite tour est restée, Raphaël. Oui, avec les cubes. Ça sent le pain, un peu tiède. Et le bois, maman. Le salon est doux, Raphaël ? Oui, papa. Le chat se couche au soleil, loin des cubes. Il dort. On laisse la tour, Raphaël ? Oui, tout près. La petite tour reste près du fauteuil. Un éclat de fauteuil tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Raphaël.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du fauteuil. Maman essuie un peu de bois. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près de la tour. Raphaël tapote le tissu du doigt. Il a une trace de soleil. Tu la vois, la trace ? Oui, maman. La petite tour est restée, Raphaël. Oui, avec les cubes. Ça sent le pain, un peu tiède. Et le bois, maman. Le salon est doux, Raphaël ? Oui, papa. Le chat se couche au soleil, loin des cubes. Il dort. On laisse la tour, Raphaël ? Oui, tout près. La petite tour reste près du fauteuil. Un &lt;emphasis level="moderate"&gt;éclat de fauteuil&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du fauteuil. Maman essuie un peu de bois. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près de la tour. Raphaël tapote le tissu du doigt. Il a une trace de soleil. Tu la vois, la trace ? Oui, maman. La petite tour est restée, Raphaël. Oui, avec les cubes. Ça sent le pain, un peu tiède. Et le bois, maman. Le salon est doux, Raphaël ? Oui, papa. Le chat se couche au soleil, loin des cubes. Il dort. On laisse la tour, Raphaël ? Oui, tout près. La petite tour reste près du fauteuil. Un &lt;emphasis&gt;éclat de fauteuil&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1993,7 +2090,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2001,10 +2098,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2013,12 +2110,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2027,17 +2124,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de fauteuil</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2046,11 +2147,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2059,27 +2160,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis triste.
-enfant-m|J'ai eu un câlin.
-papa|Pleurer est permis.
-maman|Bravo, Raphaël.</t>
+          <t>narrateur|Ils restent près du fauteuil.
+narrateur|Maman essuie un peu de bois.
+enfant-m|Les cubes sont tombés, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près de la tour.
+narrateur|Raphaël tapote le tissu du doigt.
+enfant-m|Il a une trace de soleil.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La petite tour est restée, Raphaël.
+enfant-m|Oui, avec les cubes.
+narrateur|Ça sent le pain, un peu tiède.
+enfant-m|Et le bois, maman.
+papa|Le salon est doux, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Le chat se couche au soleil, loin des cubes.
+enfant-m|Il dort.
+papa|On laisse la tour, Raphaël ?
+enfant-m|Oui, tout près.
+narrateur|La petite tour reste près du fauteuil.
+narrateur|Un éclat de fauteuil tient sur le tissu.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>chat</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2150,6 +2277,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>